<commit_message>
Copy barcodes into the Barcode field, and ask for both in the import template
The store kept every barcode in SKU and almost none in Barcode, so the
product JSON-LD (which reads Barcode for gtin) gave Google no barcode for
2,286 of 2,427 products. Done on the store on 25 Sep 2026:

- 2,054 checksum-valid barcodes copied from SKU into Barcode (2,190 now
  match; 136 already did). SKU untouched: the product page and the
  back-in-stock email still read it.
- Barcode fixed on 5: two text codes cleared, three given back the
  leading zero Excel had dropped.

barcode-changes-2026-09-25.csv logs every write with its before value.
barcode-check-2026-09-25.csv/.xlsx lists the 74 SKUs not written, grouped
by pattern and flagged for collisions and bundles, to check against the box.

The import template now asks for the barcode in both SKU and Barcodes,
and says a shop-made bundle gets no barcode.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/setup/product-import/product-import-workbook.xlsx
+++ b/setup/product-import/product-import-workbook.xlsx
@@ -209,12 +209,12 @@
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>The product's barcode (EAN, usually 13 digits). The whole store keeps the barcode here. This column is formatted as text so Excel keeps every digit.</t>
+        <t>The product's barcode (EAN, usually 13 digits). The store shows it under the title. Formatted as text so Excel keeps every digit.</t>
       </text>
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
       <text>
-        <t>Leave blank. The barcode goes in SKU.</t>
+        <t>The same barcode again, exactly as in SKU. Google reads this one.</t>
       </text>
     </comment>
     <comment ref="L1" authorId="0" shapeId="0">
@@ -612,7 +612,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>BARCODE goes in the SKU column, not the Barcodes column. That is how every product already on the store is set up. The SKU column is formatted as text so Excel does not turn 5012345678900 into 5.01E+12 or drop a leading zero.</t>
+          <t>BARCODE goes in BOTH the SKU column and the Barcodes column, the same number in each. SKU is what the product page shows; Barcodes is what Google reads. Both columns are formatted as text so Excel does not turn 5012345678900 into 5.01E+12 or drop a leading zero. A bundle made up in the shop has no barcode of its own: leave Barcodes blank rather than inventing one. (A boxed gift set from the brand has a real barcode on the box; use that.)</t>
         </is>
       </c>
     </row>
@@ -856,7 +856,11 @@
           <t>5012345678900</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr"/>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>5012345678900</t>
+        </is>
+      </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
           <t>12.99</t>
@@ -4785,7 +4789,7 @@
         </is>
       </c>
       <c r="E116" t="n">
-        <v>505</v>
+        <v>332</v>
       </c>
     </row>
     <row r="117">

</xml_diff>